<commit_message>
Leads: 2026-09-16 00:02 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://www.magnumacrepair.com/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>john@smith.com</t>
@@ -640,7 +639,6 @@
           <t>https://sunupservices.com/heating-cooling-services-st-petersburg-fl/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>customerservice@sunupservices.com</t>
@@ -670,6 +668,66 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Brown's Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>bphnh.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://bphnh.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Plumbing Specialists</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>kbrown@bphnh.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(603) 686-8109</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Manchester NH</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>88</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>plumber Manchester NH</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 00:24 UTC (cycle 195)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -733,6 +733,62 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Roof Repair Companies Lansing, MI | Elieff Brothers Roofing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>elieffbrothers.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.elieffbrothers.com/lansing-mi</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>harvey.elieff@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(517) 627-7999</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roofer Lansing MI</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 00:27 UTC (cycle 197)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -754,7 +754,6 @@
           <t>https://www.elieffbrothers.com/lansing-mi</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>harvey.elieff@gmail.com</t>
@@ -784,6 +783,66 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Corona Roof Repair</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>coronaroofrepair.homes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://coronaroofrepair.homes/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Roof Flashing</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@coronaroofrepair.homes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1951612308</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Corona CA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roof repair company Corona CA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 00:29 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -848,6 +848,242 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Houston Emergency Plumber | 24/7 Fast Response Plumbing Repair</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>houstonplumbinghelp.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://houstonplumbinghelp.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Why Houston</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>service@houstonplumbinghelp.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(832) 819-5941</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>emergency plumber Houston TX</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rapid Response Plumbing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rapidresponse-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://rapidresponse-plumbing.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Rapid Response</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>hussam@rapidresponse-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(713)-955-7140</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>emergency plumber Houston TX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Spencer's Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>spencersplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://spencersplumbingservices.com/emergency-plumbing/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>chris@spencersplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>832-658-2569</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>emergency plumber Houston TX</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rescue Plumbing &amp; HVAC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>rescueplumbingandhvac.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.rescueplumbingandhvac.com/rescue-paterson</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Read Rescue</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@rescueplumbingandhvac.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(866) 737-2830</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Paterson NJ</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>80</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>HVAC contractor Paterson NJ</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 00:32 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -989,7 +989,6 @@
           <t>https://spencersplumbingservices.com/emergency-plumbing/</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>chris@spencersplumbingservices.com</t>
@@ -1079,6 +1078,66 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Metal Roofing Katy</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>resoluteroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://resoluteroofingllc.com/areas-of-service/katy-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Commercial Roofing</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>victorb@resoluteroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(832) 498-9140</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Katy TX</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 00:33 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1143,6 +1143,66 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Young Plumbing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>youngplumbing.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.youngplumbing.com/city/gary-in/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Young Plumbing</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>service@youngplumbing.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>219.764.5500</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Gary IN</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>plumbing company Gary IN</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:18 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,62 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bonnabel Air</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>metairiecool.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://metairiecool.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>How We</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>service@metairiecool.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>86</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>air conditioning repair Metairie LA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:21 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1234,7 +1234,6 @@
           <t>service@metairiecool.com</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Metairie LA</t>
@@ -1254,6 +1253,186 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DFW Plumber</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>dfwplumber.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.dfwplumber.com/plumbers/emergency-plumbers-dallas/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Reach Out</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>service@dfwplumber.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(214) 334-3424</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>emergency plumber Dallas TX</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Texas Slab Leaks LLC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>texasslableaksrepair.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://texasslableaksrepair.com/emergency-plumbing-in-dallas/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Local Family</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>bluem9817@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(469)-352-6031</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>emergency plumber Dallas TX</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Holy City Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>holycityhvac.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.holycityhvac.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Homeowner Education</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@holycityhvac.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(843) 790-6504</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Charleston SC</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>AC installation Charleston SC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:22 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1438,6 +1438,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Promar Roofing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>promarroofing.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://promarroofing.com/home-metal-roof/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Unique Benefits</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@promarroofing.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(847) 999-1309</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Chicago IL</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:24 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1498,6 +1498,122 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Anthony Brothers Water Heaters</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>anthonybrothers.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.anthonybrothers.com/locations/hollywood</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Story Anthony</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@anthonybrothersplumbing.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(954) 516-6755</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>water heater repair Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Atchley Air Cooling, Heating, Plumbing &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>atchleyair.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://atchleyair.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>service@atchleyair.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(479) 207-6862</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Fort Smith AR</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fort Smith AR</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:27 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1579,7 +1579,6 @@
           <t>https://atchleyair.com/</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>service@atchleyair.com</t>
@@ -1609,6 +1608,66 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Complete Roofing</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>completeroofco.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://completeroofco.com/locations/greater-new-orleans-residential-commercial-roofing/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Nathan Sisk</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@completeroofco.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(228) 202-5542</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>residential roofing company New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:28 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1673,6 +1673,66 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HVAC &amp; Electrical Services Houston, TX | TL Techs</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>tltechs.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://tltechs.com/location/sugar-land-tx/hvac-services-sugar-land/ac-installation-sugar-land/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Tony Doan</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>tltechsco@gmail.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>832-430-9042</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>84</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>AC installation Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:30 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1733,6 +1733,122 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>B&amp;B</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>bbheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.bbheatingcooling.com/locations/ofallon/air-conditioning-repair-ofallon/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>bbhvac1955@gmail.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>314-668-8530</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>air conditioning repair OFallon MO</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>KirbnJays Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>kirbnjayshvac.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.kirbnjayshvac.com/services/air-conditioning-repair</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Ownership Stand</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>jason@kirbnjayshvac.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(636) 747-1667</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>air conditioning repair OFallon MO</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:34 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1754,7 +1754,6 @@
           <t>https://www.bbheatingcooling.com/locations/ofallon/air-conditioning-repair-ofallon/</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>bbhvac1955@gmail.com</t>
@@ -1844,6 +1843,66 @@
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Flo Mechanical Solutions</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>fmsut.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://fmsut.com/residential/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Salt Lake</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>service@fmsut.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(801) 871-5217</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>84</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>furnace repair Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:44 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1908,66 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Rancho Cucamonga</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>rancho-cucamonga-ca.metalproroofingarcadia.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://rancho-cucamonga-ca.metalproroofingarcadia.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>info@metalproroofingarcadia.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(833) 642-0267</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>90</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:46 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1968,6 +1968,62 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bend Plumbing Pros | Plumbing Service Bend Oregon</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>bendplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://bendplumbingpros.com/service/emergency-plumbing/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>randy@besttownagents.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(541) 844-4880</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>90</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>emergency plumber Bend OR</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:47 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1989,7 +1989,6 @@
           <t>https://bendplumbingpros.com/service/emergency-plumbing/</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>randy@besttownagents.com</t>
@@ -2019,6 +2018,122 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Roof Construction Eugene, OR</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>eugeneroofconstruction.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.eugeneroofconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Repair Roof</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>eugenegeneralconstruction@gmail.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>541788-6836</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Eugene OR</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>roofing contractor Eugene OR</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>O'Connor Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>oconnorhvacscia.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://oconnorhvacscia.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>pochvac@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>712-490-7827</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Sioux City IA</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>90</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>heating and cooling company Sioux City IA</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:49 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2104,7 +2104,6 @@
           <t>https://oconnorhvacscia.com/</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>pochvac@hotmail.com</t>
@@ -2134,6 +2133,62 @@
         </is>
       </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Coza Crew Plumbing</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>cozacrewplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.cozacrewplumbingllc.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@cozacrewplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>854-295-7895</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Summerville SC</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>84</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>plumbing company Summerville SC</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:57 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2159,7 +2159,6 @@
           <t>https://www.cozacrewplumbingllc.com/</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>info@cozacrewplumbingllc.com</t>
@@ -2189,6 +2188,242 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PureFlo Plumbing</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>purefloplumbingjax.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://purefloplumbingjax.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Jobs Big</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>contact@pureflo-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>904-803-0495</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>100</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>plumbing company Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Water Heater Pasadena, TX</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>waterheaterpasadenatx.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://waterheaterpasadenatx.com/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>service@waterheaterpasadenatx.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>281-402-9243</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>water heater repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Hot Water Heaters</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>hotwaterheaterstx.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://hotwaterheaterstx.com/pasadenatx.html</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Business Owner</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>service@hotwaterheaterstx.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>281-643-7103</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>94</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>water heater repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SOS Water Heater Pasadena TX</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>pasadena.soswaterheater.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://pasadena.soswaterheater.com/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Questions Answered</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>service@pasadena.soswaterheater.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>346-569-8179</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>92</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>water heater repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 13:59 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2274,7 +2274,6 @@
           <t>https://waterheaterpasadenatx.com/</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>service@waterheaterpasadenatx.com</t>
@@ -2424,6 +2423,66 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Exterior Building Solutions (EBS) Roofing, Siding, &amp; Windows</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>exteriorbuildingsolutions.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://exteriorbuildingsolutions.com/areas-we-serve/ofallon-mo</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Building Solutions</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>info@exteriorbuildingsolutions.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(314) 729-7663</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>OFallon MO</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>roof replacement OFallon MO</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:00 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2488,6 +2488,62 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>FES Roofing</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>fesroofing.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.fesroofing.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>allen@fesroofing.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(479) 275-5332</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>90</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>residential roofing company Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:05 UTC (cycle 33)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2509,7 +2509,6 @@
           <t>https://www.fesroofing.com/</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>allen@fesroofing.com</t>
@@ -2539,6 +2538,66 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in West Palm Beach, FL - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>westpalmbeachhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://westpalmbeachhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Rosemary Ave</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>info@westpalmbeachhvacpros.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(561) 677-5933</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>100</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>heating and cooling company West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:06 UTC (cycle 34)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2603,6 +2603,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>pictureperfectexteriors</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>pictureperfectexteriors.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://pictureperfectexteriors.com/roofing/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Perfect Exteriors</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>info@pictureperfectexteriors.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>412-743-8208</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>100</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:12 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2663,6 +2663,62 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DM Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>dmroofing.org</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://dmroofing.org/southaven-mississippi/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>david@dmroofing.org</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(901) 356-9292</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Southaven MS</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>90</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>residential roofing company Southaven MS</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:19 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2684,7 +2684,6 @@
           <t>https://dmroofing.org/southaven-mississippi/</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>david@dmroofing.org</t>
@@ -2714,6 +2713,62 @@
         </is>
       </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Roofing Brooklyn</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>roofingbrooklyn.co</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://roofingbrooklyn.co/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>hi@roofingbrooklyn.co</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(929) 595-7756</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>100</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>roofing contractor Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:22 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2739,7 +2739,6 @@
           <t>https://roofingbrooklyn.co/</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>hi@roofingbrooklyn.co</t>
@@ -2769,6 +2768,62 @@
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Top Quality Plumbers | Rooter Man Plumbing | Reno Carson | Best Plumbers In Reno</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>rootermanrenocarson.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://rootermanrenocarson.com/sewer-repair-reno-nv/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>rootermanffice1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>775-624-3324</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Reno NV</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>80</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>sewer repair Reno NV</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:25 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2794,7 +2794,6 @@
           <t>https://rootermanrenocarson.com/sewer-repair-reno-nv/</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>rootermanffice1@gmail.com</t>
@@ -2824,6 +2823,62 @@
         </is>
       </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Colorado Bear Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>cobearhvac.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.cobearhvac.com/heat-pump/heat-pump-installation-replacement-aurora-co</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>support@cobearhvac.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(720) 790-3765</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>heat pump installation Aurora CO</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:31 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2849,7 +2849,6 @@
           <t>https://www.cobearhvac.com/heat-pump/heat-pump-installation-replacement-aurora-co</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>support@cobearhvac.com</t>
@@ -2879,6 +2878,66 @@
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>The Prull Group | Top Professional Heating &amp; Cooling Contractor</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>prullgroup.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://prullgroup.com/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Careers Contact</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>projects@prullgroup.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(319) 826-1074</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>90</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>HVAC contractor Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:33 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2943,6 +2943,126 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Benchmark Air â Tampa, Clearwater &amp; St. Petersburg heating and cooling</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>benchmarkairfl.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://benchmarkairfl.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Tampa Bay</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>careers@benchmarkair.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(813) 555-0142</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>100</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>heating and cooling company Tampa FL</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Royal King Plumbing - Clearwater plumber serving Pinellas County, Pasco County a</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>royalkingplumbing.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://royalkingplumbing.com/service-areas/pinellas-county/clearwater/emergency-plumber/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>King Plumbing</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>info@royalkingplumbing.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>800-990-6514</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>emergency plumber Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:34 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3063,6 +3063,122 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sky Heating</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>skyheating.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://skyheating.com/hvac-services/ac-replacement/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>csrleads@skyheating.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(503) 563-2698</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>100</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>AC installation Portland OR</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Complete Climate Services</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>completeclimateservices.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.completeclimateservices.com/services/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>View All</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@completeclimateservices.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>443-898-4747</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>furnace repair Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:36 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3084,7 +3084,6 @@
           <t>https://skyheating.com/hvac-services/ac-replacement/</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>csrleads@skyheating.com</t>
@@ -3174,6 +3173,62 @@
         </is>
       </c>
       <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>HVAC STANDARD</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>hvac-standard.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.hvac-standard.com/professional-fast-ac-installation-mount-vernon-ny/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>contact@casse-auto.veri-couvreur.fr</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>646 828 9914</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>90</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>AC installation Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:39 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3199,7 +3199,6 @@
           <t>https://www.hvac-standard.com/professional-fast-ac-installation-mount-vernon-ny/</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>contact@casse-auto.veri-couvreur.fr</t>
@@ -3229,6 +3228,126 @@
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Long Home</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>longhome.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://longhome.com/locations/maryland/waldorf/roofing/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Future As</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>info@longhome.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(800) 417-5664</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Waldorf MD</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>roof replacement Waldorf MD</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Addario's Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>plumberlowellma.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.plumberlowellma.com/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Plumbing Services</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>info@plumberlowellma.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(831) 204-4288</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Lowell MA</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>90</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>plumber Lowell MA</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:40 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3353,6 +3353,122 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Gibbs Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>goingwithgibbs.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://goingwithgibbs.com/services/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>At Gibbs</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>info@goingwithgibbs.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(404) 545-6900</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>100</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>roof replacement Roswell GA</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>AirPro Heating, Cooling &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>okairpro.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://okairpro.com/broken-arrow-ok/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>shanehvac1980@gmail.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(918) 543-1400</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>AC installation Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:46 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3434,7 +3434,6 @@
           <t>https://okairpro.com/broken-arrow-ok/</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>shanehvac1980@gmail.com</t>
@@ -3464,6 +3463,122 @@
         </is>
       </c>
       <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>plumbingmckinney-tx.com</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>plumbingmckinney-tx.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://plumbingmckinney-tx.com/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>service@plumbingmckinney-tx.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>469-665-9414</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>100</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>plumbing company McKinney TX</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Elite Construction &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>eliteconstructionandroofing.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://eliteconstructionandroofing.com/service-areas/boulder-co/metal-roofs/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>At Elite</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>office@elitesc.net</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(720) 794-8574</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Boulder CO</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>90</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Boulder CO</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 14:52 UTC (cycle 65)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3489,7 +3489,6 @@
           <t>https://plumbingmckinney-tx.com/</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>service@plumbingmckinney-tx.com</t>
@@ -3579,6 +3578,122 @@
         </is>
       </c>
       <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Markopoulos Roofing</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>markopoulosroofing.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://markopoulosroofing.com/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Read More</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>info@markopoulosroofing.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(774) 437-2313</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>98</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>roof repair company Worcester MA</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>R3 Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>r3hvac.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://r3hvac.com/heating-in-davenport-iowa/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>info@r3mech.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>309-232-8774</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>furnace repair Davenport IA</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:06 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3664,7 +3664,6 @@
           <t>https://r3hvac.com/heating-in-davenport-iowa/</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>info@r3mech.com</t>
@@ -3694,6 +3693,62 @@
         </is>
       </c>
       <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Rod's Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>rodsplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.rodsplumbingservice.com/water-heaters-fresno</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>rod@rodsplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>(559) 388-2600</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>90</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>water heater repair Fresno CA</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:18 UTC (cycle 83)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3719,7 +3719,6 @@
           <t>https://www.rodsplumbingservice.com/water-heaters-fresno</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>rod@rodsplumbingservice.com</t>
@@ -3749,6 +3748,126 @@
         </is>
       </c>
       <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Green Quest Roofing - Virginia Commercial Roofing Company</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>greenquestroofing.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://greenquestroofing.com/metal-roofing-fredericksburg-va/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Eli Kinsinger</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>sales@greenquestroofing.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(877) 576-6396</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>96</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>King Roofing &amp; Construction, LLC</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>kingroofingva.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://kingroofingva.com/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Contractors License</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>brendan@kingroofingva.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(703) 932-0354</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>84</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:21 UTC (cycle 85)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3873,6 +3873,66 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Jordan River Roofing</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>jordanriverroofing.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.jordanriverroofing.com/areas-we-serve/west-jordan-ut/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Serve You</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>johnsmith@gmail.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(801) 857-1417</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>West Jordan UT</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>90</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>roof replacement West Jordan UT</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:28 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3933,6 +3933,62 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Elevation Roofing</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>elevationroofingnm.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.elevationroofingnm.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>elevationroofingcompany@gmail.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>505-980-9706</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>68</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:36 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3954,7 +3954,6 @@
           <t>https://www.elevationroofingnm.com/metal-roofing</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>elevationroofingcompany@gmail.com</t>
@@ -3984,6 +3983,66 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Best Norman Plumbers</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>norman-plumber.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://norman-plumber.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Pros Locally</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>sales@veteranplumbing.net</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(405) 818-0467</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Norman OK</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>90</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>plumber Norman OK</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:39 UTC (cycle 97)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4048,6 +4048,62 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Bluefin Exteriors LLC</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>bluefinroof.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://bluefinroof.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Coatings Roof</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>office@bluefinroof.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>86</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>roof repair company Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:40 UTC (cycle 98)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4079,7 +4079,6 @@
           <t>office@bluefinroof.com</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>Tuscaloosa AL</t>
@@ -4099,6 +4098,62 @@
         </is>
       </c>
       <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Orlando Roofing</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>theorlandoroofingco.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://theorlandoroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>admin@theorlandoroofingco.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(407) 275-9444</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>96</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>residential roofing company Orlando FL</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:43 UTC (cycle 100)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4124,7 +4124,6 @@
           <t>https://theorlandoroofingco.com/</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>admin@theorlandoroofingco.com</t>
@@ -4154,6 +4153,126 @@
         </is>
       </c>
       <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Pasadena, TX | Sentry Pro Roofing</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>sentryproroofingl.shop</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://sentryproroofingl.shop/service-areas/pasadena-tx</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Katy Fwy</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>info@sentryproroofingl.shop</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(209) 758-8550</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>roofing contractor Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Plumber Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>plumberpalmbayfl.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>http://plumberpalmbayfl.com/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Why Brevard</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>service@plumberpalmbayfl.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(321) 404-1946</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>78</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>emergency plumber Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:49 UTC (cycle 104)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4278,6 +4278,66 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in McKinney, TX - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>mckinneyhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://mckinneyhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Service Areas</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>info@mckinneyhvacpros.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(214) 751-8830</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>HVAC contractor McKinney TX</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:53 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4338,6 +4338,66 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Jersey City NJ HVAC Contractor | AC &amp; Heat Pump Installation | Up to $16K Rebate</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>mechanicalenterprise.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://mechanicalenterprise.com/hvac-jersey-city-nj</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>info@mechanicalenterprise.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(862) 423-9396</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>100</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>heat pump installation Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:56 UTC (cycle 109)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4398,6 +4398,66 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Top Line Roofing Contractors</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>toplineroofingcontractors.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.toplineroofingcontractors.com/portland-or/metal-roofing-portland/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Owner Scott</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>toplineroofingcontractors1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(503) 206-3167</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>100</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Portland OR</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:58 UTC (cycle 110)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4458,6 +4458,122 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Macon, GA - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>maconacrepair.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://maconacrepair.com/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Luther King</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>info@maconacrepair.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(478) 812-6012</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Macon GA</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>100</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>heating and cooling company Macon GA</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>All American Roofing</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>allamericanroofingkc.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://www.allamericanroofingkc.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>tmp488@gmail.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>913-345-8000</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>96</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>roofer Olathe KS</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 15:59 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4539,7 +4539,6 @@
           <t>https://www.allamericanroofingkc.com/</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>tmp488@gmail.com</t>
@@ -4569,6 +4568,66 @@
         </is>
       </c>
       <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Stinson Services</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>stinsonservices.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://stinsonservices.com/brooklyn-park/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Stinson Services</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>contact@stinsonservices.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>952-933-4510</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>residential roofing company Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:09 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4633,6 +4633,62 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Home | Evergreen Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>evergreenhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://www.evergreenhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>info@evergreenhvacpros.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(555) 555-5555</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Lafayette IN</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>furnace repair Lafayette IN</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:14 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4654,7 +4654,6 @@
           <t>https://www.evergreenhvacpros.com/</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>info@evergreenhvacpros.com</t>
@@ -4684,6 +4683,66 @@
         </is>
       </c>
       <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Academy Roofing</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>academyroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.academyroofinginc.com/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Academy Roofing</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>estimates@academyroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>303.360.0708</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>96</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>roofer Aurora CO</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:15 UTC (cycle 122)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4748,6 +4748,122 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Boston Drain Service</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>bostondrainservices.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://bostondrainservices.com/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>info@bostondrainservices.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>617-286-5670</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>86</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>drain cleaning service Boston MA</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Boston Drain Pros</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>bostondrainpros.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.bostondrainpros.com/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>North Shore</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>info@bostondrainpros.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(781) 205-0392</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>74</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>drain cleaning service Boston MA</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:21 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4769,7 +4769,6 @@
           <t>https://bostondrainservices.com/</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>info@bostondrainservices.com</t>
@@ -4859,6 +4858,126 @@
         </is>
       </c>
       <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Sarasota, Manatee &amp; Charlotte Counties | SonShine Roofing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>sonshineroofing.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://sonshineroofing.com/roof-replacement-sarasota-fl</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Team Nathan</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>messages@sonshineroofing.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(941) 866-4320</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>90</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>roof replacement Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Panda Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>pandaheating.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://www.pandaheating.com/service-areas/mckinney-tx/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Reviews What</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>support@pandaheating.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>469-919-7646</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>90</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>furnace repair McKinney TX</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:23 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4983,6 +4983,66 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Right Away Sewer &amp; Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>rightawaysewercleaning.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://rightawaysewercleaning.com/residential/brooklyn-park/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>St Paul</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>office@rightawaysewercleaning.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(612) 545-8483</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>90</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>drain cleaning service Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:40 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5043,6 +5043,66 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>United Construction &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>unitedconstructionroofing.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.unitedconstructionroofing.com/areas-we-serve/hillsboro-or-roofer/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Heather See</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>user@gmail.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(971) 379-7163</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>100</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>roof repair company Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:57 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5103,6 +5103,122 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>B &amp; M Roofing</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>bandmroofing.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://bandmroofing.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Built From</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>contact@bandmroofing.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>520-460-5331</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>86</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>residential roofing company Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Molnar Air - Lakeland Air Conditioning Contractor</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>molnarair.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://molnarair.com/lakeland-hvac-contractor/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>info@molnarair.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>863-333-4916</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>80</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>HVAC contractor Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 16:59 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5184,7 +5184,6 @@
           <t>https://molnarair.com/lakeland-hvac-contractor/</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>info@molnarair.com</t>
@@ -5214,6 +5213,62 @@
         </is>
       </c>
       <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Complete Comfort Air</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>completecomfortair.net</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://completecomfortair.net/air-conditioning/ac-installation-in-columbia/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>service@completecomfortair.net</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>(803) 862-7194</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>90</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>AC installation Columbia SC</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 17:02 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5239,7 +5239,6 @@
           <t>https://completecomfortair.net/air-conditioning/ac-installation-in-columbia/</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>service@completecomfortair.net</t>
@@ -5269,6 +5268,66 @@
         </is>
       </c>
       <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Furnace Doctors Inc.</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>furnacedoctors.org</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://furnacedoctors.org/hvac/renton-wa/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Furnace Doctors</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>johnfurnacedoc@aol.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(206) 622-5018</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Renton WA</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>90</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>furnace repair Renton WA</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 17:03 UTC (cycle 155)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5333,6 +5333,182 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Superb Roofing &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>superbroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://superbroofingllc.com/services/roof-repair-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>From Roofer</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>info@superbroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(830) 251-4852</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>roof replacement New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>NEW BRAUNFELS ROOFING</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>newbraunfelsroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.newbraunfelsroofingtx.com/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>New Braunfels</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>info@newbraunfelsroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>(830) 542-8333</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>90</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>roof replacement New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Roof Replacement in New Braunfels</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>arroyosroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://arroyosroofingllc.com/locations/new-braunfels-tx/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>info@arroyosroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(833) 747-0551</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>roof replacement New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 17:19 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5474,7 +5474,6 @@
           <t>https://arroyosroofingllc.com/locations/new-braunfels-tx/roof-replacement</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>info@arroyosroofingllc.com</t>
@@ -5504,6 +5503,62 @@
         </is>
       </c>
       <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>True Colors Industrial, LLC</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>metalroofsouthbend.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>http://www.metalroofsouthbend.com/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofsouthbend.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(888) 862-5043</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>South Bend IN</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>84</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>metal roofing contractor South Bend IN</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 17:21 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5529,7 +5529,6 @@
           <t>http://www.metalroofsouthbend.com/</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>moreinfo@metalroofsouthbend.com</t>
@@ -5559,6 +5558,66 @@
         </is>
       </c>
       <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Residential Roofing &amp; Solar Services | San Diego County | Dils Roofing</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>dilsroofing.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.dilsroofing.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>customerservice@dilsroofing.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(760) 727-6000</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>100</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>roof repair company San Diego CA</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 17:39 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5623,6 +5623,66 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>HVAC Contractor in Naperville, IL | FortHouse</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forthousehvac.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.forthousehvac.com/hvac-naperville-il</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Jenna Fortman</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>comfort@forthousehvac.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(630) 318-6246</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>100</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>HVAC contractor Naperville IL</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 17:45 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5683,6 +5683,66 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>AirPro Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>airproky.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://www.airproky.com/ac-installation-lexington-ky/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Igor Reznichenko</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>airpro.ky@gmail.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>859-490-0258</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>90</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>AC installation Lexington KY</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 17:48 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5743,6 +5743,66 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Juan &amp; Only Plumber</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>juanandonlyplumber.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://juanandonlyplumber.com/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>All Testimonial</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>info@juanandonlyplumber.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(512) 222-7311</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>90</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>plumber Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 18:00 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5803,6 +5803,122 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>E Dennis</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>edennisacinc.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://edennisacinc.com/hvac-sandy-springs/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Heritage Park</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>info@edennisacinc.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(770) 758-0501</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>100</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>furnace repair Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Doty Service Network - Experience the Doty Difference</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>dotymechanical.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://dotymechanical.com/</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>info@dotymechanical.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(517) 327-7777</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>90</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>furnace repair Lansing MI</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 18:05 UTC (cycle 197)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5884,7 +5884,6 @@
           <t>https://dotymechanical.com/</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>info@dotymechanical.com</t>
@@ -5914,6 +5913,62 @@
         </is>
       </c>
       <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Midway Sewer &amp; Pumping Service Residential &amp; Commercial</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>midwaysewer.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.midwaysewer.com/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>midwaysewer@aol.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(218) 628-0345</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>94</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>sewer repair Duluth MN</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 18:06 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5939,7 +5939,6 @@
           <t>https://www.midwaysewer.com/</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>midwaysewer@aol.com</t>
@@ -5969,6 +5968,66 @@
         </is>
       </c>
       <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>American Contracting Team LLC</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>americancontractingteam.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.americancontractingteam.com/edison-nj.html</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>americancontractingteam@gmail.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(848) 391-1251</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Edison NJ</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>100</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>roofing contractor Edison NJ</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 18:16 UTC (cycle 205)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6033,6 +6033,182 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Heating Repair in Miramar, FL - 24/7 Emergency Service</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>koolflowair.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://koolflowair.com/heating/heating-repair-miramar-fl</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>service@koolflowair.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(954) 962-8843</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>100</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>furnace repair Miramar FL</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Florida 5 Star Roofing | Central Florida's Premier Roofing Services Company</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>fl5starroofing.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.fl5starroofing.com/kissimmee/</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Osceola County</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>office@fl5starroofing.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(407) 634-3335</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>100</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>residential roofing company Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Noland's Roofing</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>nolandsroofing.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://nolandsroofing.com/locations/kissimmee</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Osceola County</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>customerservice@nolandsroofing.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(352) 242-4322</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>90</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>residential roofing company Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 18:18 UTC (cycle 206)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6054,7 +6054,6 @@
           <t>https://koolflowair.com/heating/heating-repair-miramar-fl</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>service@koolflowair.com</t>
@@ -6204,6 +6203,122 @@
         </is>
       </c>
       <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Johns Plumbing</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>johnsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://johnsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>info@johnsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(954) 923-4184</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>90</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>drain cleaning service Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>CEC Plumbing, Inc.</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>cecplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.cecplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Sewer Now</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>admin@covertmarketing.agency</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(954) 791-2327</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>90</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>drain cleaning service Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:28 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6229,7 +6229,6 @@
           <t>https://johnsplumbing.com/</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>info@johnsplumbing.com</t>
@@ -6319,6 +6318,122 @@
         </is>
       </c>
       <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>HomeServe of Staten Island</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>homeservesi.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.homeservesi.com/cooling/air-conditioning-installation/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>david.johnson@strategicamerica.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(888) 211-0578</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Staten Island NY</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>100</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>AC installation Staten Island NY</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Green Roofing Chicago</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>greenroofingchicago.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://greenroofingchicago.com/residential-roofing-chicago-il/</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Saying About</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>info@greenroofingchicago.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(312) 428-7504</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>90</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>residential roofing company Chicago IL</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:29 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6344,7 +6344,6 @@
           <t>https://www.homeservesi.com/cooling/air-conditioning-installation/</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>david.johnson@strategicamerica.com</t>
@@ -6434,6 +6433,66 @@
         </is>
       </c>
       <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>HVAC Company | Waukesha, WI | Tom's Heating Service LLC</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>tomsheating.net</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.tomsheating.net/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Read More</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>melissa@tomsheating.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(262) 548-1300</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Waukesha WI</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>90</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>heating and cooling company Waukesha WI</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:32 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6498,6 +6498,246 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Dearborn Plumbing Pro</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>dearbornplumbingpro.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://dearbornplumbingpro.com/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Michigan Ave</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>info@dearbornplumbingpro.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(313) 251 4847</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Dearborn MI</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>100</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>plumber Dearborn MI</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>HVAC Company Missouri</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>heat-pump-installation-springfield.heatingcoolingmacon.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://heat-pump-installation-springfield.heatingcoolingmacon.com/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Call Now</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>admin@sood.heritageplumbinggrantspass.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>(888) 709-2550</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Springfield MO</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>100</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>heat pump installation Springfield MO</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>New Generation Roofing</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>newgeneration-roofing.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.newgeneration-roofing.com/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Menu Home</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>newgenerationroof@gmail.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>503-519-6421</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Gresham OR</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>100</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>roof replacement Gresham OR</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>A Plus Plumbers Federal Way</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>aplusplumbersfederalway.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.aplusplumbersfederalway.com/drain-services-federal-way-wa/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Federal Way</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>info@aplusplumbersfederalway.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(253) 264 0803</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>90</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>drain cleaning service Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:34 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6738,6 +6738,126 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>MQ Roofing | The Best Protection for Your Investment!</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>mqroofing.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.mqroofing.com/metal-roofers-appleton-wi/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Coated Steel</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@mqroofing.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(608) 553-3300</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Appleton WI</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>100</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Appleton WI</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Metal Roofing Appleton WI | Anytime Roofing</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>anytimeroofingwi.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://anytimeroofingwi.com/service-areas/appleton-wi</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>See Why</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>ray@anytimeroofingwi.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>6087210940</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Appleton WI</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>90</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Appleton WI</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:35 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6858,6 +6858,66 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>AccuFlow Plumbing, Inc.</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>accuflowplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://accuflowplumbinginc.com/service-area/stockton.html</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Frequently Asked</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>info@accuflowplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>(209) 330-3569</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>100</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>plumbing company Stockton CA</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:40 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6918,6 +6918,66 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Sewer23™ -</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>sewer23.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://sewer23.com/locations/dearborn/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Expertise You</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>service@sewer23.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>248-993-3423</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Dearborn MI</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>90</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>sewer repair Dearborn MI</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:41 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6978,6 +6978,66 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Roof Gutter Now</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>roofgutternow.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://roofgutternow.com/locations/ohio/youngstown/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Gutter Now</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@roofgutternow.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(330) 918-1018</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Youngstown OH</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>100</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>roof repair company Youngstown OH</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:46 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7038,6 +7038,118 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>KPS Plumbing</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>kpsplumbing.co</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://kpsplumbing.co/sewer/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>joel@kpsplumbing.co</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>661-817-0637</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>100</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>sewer repair Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Roofing Contractors Harrisburg Pa</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>roofingcontractorsharrisburgpa.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://roofingcontractorsharrisburgpa.com/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>hello@rfuenzalida.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>888-837-5857</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>76</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>roofing contractor Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:47 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7059,7 +7059,6 @@
           <t>https://kpsplumbing.co/sewer/</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>joel@kpsplumbing.co</t>
@@ -7115,7 +7114,6 @@
           <t>https://roofingcontractorsharrisburgpa.com/</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>hello@rfuenzalida.com</t>
@@ -7145,6 +7143,118 @@
         </is>
       </c>
       <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>HVAC Services | C &amp; C Temp Control | Worcester &amp; Auburn, MA</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>cctempcontrol.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://www.cctempcontrol.com/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>bob@cctempcontrol.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>(508) 853-7900</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>heating and cooling company Worcester MA</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Chaves Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>chaveshvac.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://www.chaveshvac.com/city/worcester-ma/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>andre@chaveshvac.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>978-562-5309</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>90</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>heating and cooling company Worcester MA</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:48 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7169,7 +7169,6 @@
           <t>https://www.cctempcontrol.com/</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>bob@cctempcontrol.com</t>
@@ -7225,7 +7224,6 @@
           <t>https://www.chaveshvac.com/city/worcester-ma/</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>andre@chaveshvac.com</t>
@@ -7255,6 +7253,62 @@
         </is>
       </c>
       <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Mysite</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>pineappleairaz.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://www.pineappleairaz.com/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>info@pineappleairaz.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(480) 310 0240</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>100</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>air conditioning repair Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:50 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7279,7 +7279,6 @@
           <t>https://www.pineappleairaz.com/</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>info@pineappleairaz.com</t>
@@ -7309,6 +7308,62 @@
         </is>
       </c>
       <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Roofing Specialists Northwest</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>roofingspecialistsnw.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://roofingspecialistsnw.com/roofing-renton</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>info@roofingspecialistsnw.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>(425) 741-3744</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Renton WA</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>roof replacement Renton WA</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:56 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7334,7 +7334,6 @@
           <t>https://roofingspecialistsnw.com/roofing-renton</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>info@roofingspecialistsnw.com</t>
@@ -7364,6 +7363,126 @@
         </is>
       </c>
       <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Harper Roofing: Expert Roof Replacement &amp; Repair in Lakeland &amp; Central Florida</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>harperroofingfl.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://harperroofingfl.com/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Across Central</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>harperroofingfl@gmail.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>(863)-250-7663</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>90</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>roof replacement Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Expert Roof Replacements - Roofing King Lakeland, FL</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>roofingkingflorida.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://roofingkingflorida.com/roof-replacements</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Your Kingdom</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>roofingkingflorida@gmail.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(863) 670-8517</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>roof replacement Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 19:59 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7488,6 +7488,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation &amp; Replacement in Denver, CO | Elite HVAC Co</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>elitehvacco.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://elitehvacco.com/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Why Denver</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>elitehvaccorp@gmail.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(720) 806-4774</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Denver CO</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>90</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>heat pump installation Denver CO</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:00 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7548,6 +7548,66 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ASAP Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>asaproofing.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://asaproofing.com/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Joseph Kozel</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>email@asaproofing.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(903) 363-9160</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Tyler TX</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>100</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>roof repair company Tyler TX</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:06 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7608,6 +7608,62 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Oxnard Plumbing Pro</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>oxnardplumbingpro.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://oxnardplumbingpro.com/drain-cleaning-oxnard-ca/</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>info@oxnardplumbingpro.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(805) 833-5409</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Oxnard CA</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>90</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>drain cleaning service Oxnard CA</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:10 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7629,7 +7629,6 @@
           <t>https://oxnardplumbingpro.com/drain-cleaning-oxnard-ca/</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>info@oxnardplumbingpro.com</t>
@@ -7659,6 +7658,62 @@
         </is>
       </c>
       <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Reno Plumbing Doctor|Water Heater Repair</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>renowaterheaterrepair.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://www.renowaterheaterrepair.com/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>jeri@renoplumbingdoctor.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>775-852-0111</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Reno NV</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>84</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>water heater repair Reno NV</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:13 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7684,7 +7684,6 @@
           <t>https://www.renowaterheaterrepair.com/</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>jeri@renoplumbingdoctor.com</t>
@@ -7714,6 +7713,122 @@
         </is>
       </c>
       <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>McCray Roofing</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>mccrayroofing.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://mccrayroofing.com/service-areas/mclennan-county-tx/waco/</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>What Central</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>luke@mccraycg.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>254-760-6358</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Waco TX</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>100</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Waco TX</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Benson and Falgout, LLC</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>metalroofwacotx.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://metalroofwacotx.com/</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofwacotx.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>254-410-0191</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Waco TX</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>96</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Waco TX</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:15 UTC (cycle 33)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7799,7 +7799,6 @@
           <t>https://metalroofwacotx.com/</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>moreinfo@metalroofwacotx.com</t>
@@ -7829,6 +7828,62 @@
         </is>
       </c>
       <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Kessler Roofing</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>kesslerroofing.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://www.kesslerroofing.com/service-areas/fort-collins-roofers.html</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>kesslerroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>970-667-6850</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>90</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>roofer Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:21 UTC (cycle 37)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7854,7 +7854,6 @@
           <t>https://www.kesslerroofing.com/service-areas/fort-collins-roofers.html</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>kesslerroofing@gmail.com</t>
@@ -7884,6 +7883,242 @@
         </is>
       </c>
       <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Greenville Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>metalroofinggreenville.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://metalroofinggreenville.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Message From</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>go@ccteam.org</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>(864) 259-1707</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>100</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greenville SC</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>SureFlow Roofing - Roofers in Seneca SC</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>sureflowroof.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://sureflowroof.com/greenville-sc-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Noise During</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>sureflowroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>(864) 903-7873</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>90</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greenville SC</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Tip Top Roofing LLC: Trusted roofing experts in Jonesboro, Arkansas</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>tiptoproofingusa.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://www.tiptoproofingusa.com/</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>nicholas@tiptoproofingusa.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(870) 343-9300</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>90</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>residential roofing company Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Allcon Roofing in Greenville, SC</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>allconroofing.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://www.allconroofing.com/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Craig Perfect</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>sales@allconroofing.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(864) 552-1365</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>90</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greenville SC</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:28 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8029,7 +8029,6 @@
           <t>https://www.tiptoproofingusa.com/</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>nicholas@tiptoproofingusa.com</t>
@@ -8119,6 +8118,66 @@
         </is>
       </c>
       <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Heating and Cooling Services | Hartford, CT | Ortiz Refrigeration A/C &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>ortizrefrigerationacandheatingllc.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://www.ortizrefrigerationacandheatingllc.com/hartford-ct/heating-and-cooling-services</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Maintenance Tips</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>anao@ortizhvacr.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>860-799-6283</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Hartford CT</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>96</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>heating and cooling company Hartford CT</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:32 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8183,6 +8183,66 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation | Northern NJ</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>climaxheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://www.climaxheatingandcooling.com/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>climaxnj@gmail.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>(862) 212-3847</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Newark NJ</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>100</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>heat pump installation Newark NJ</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:41 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8243,6 +8243,126 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Find Roofing Pros</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>findroofingpros.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.findroofingpros.com/lehi/roofing-contractor</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Dashboard Get</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>daniel@findroofingpros.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(801) 341-8071</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Lehi UT</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>100</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>roofing contractor Lehi UT</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Lehi, UT | Epic Roofing Contractors</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>epicroofingutah.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://epicroofingutah.com/service-areas/lehi</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Utah County</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>epicroofing.utah@gmail.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(385) 200-4040</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Lehi UT</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>88</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>roofing contractor Lehi UT</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:43 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:L137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8363,6 +8363,66 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Team Mechanical</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>teammechanical.net</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://teammechanical.net/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Installation Maintenance</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>mcarlson@teammechanical.net</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>(612) 729-5646</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>90</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>HVAC contractor Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:47 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L137"/>
+  <dimension ref="A1:L138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8423,6 +8423,58 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>LocalSpark®</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>localspark.com</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://localspark.com/best-heating-and-cooling-companies-in-honolulu-hi/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>support@localspark.com</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>86</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>heating and cooling company Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:49 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L138"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8444,13 +8444,11 @@
           <t>https://localspark.com/best-heating-and-cooling-companies-in-honolulu-hi/</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>support@localspark.com</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
           <t>Honolulu HI</t>
@@ -8470,6 +8468,122 @@
         </is>
       </c>
       <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>TNT Service Group</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>tntservicegroup.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://tntservicegroup.com/plumbing-services/sewer-lines/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Live Oaks</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>service@tnt.jdpps.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>(912) 549-1521</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Savannah GA</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>96</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>sewer repair Savannah GA</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Edwards Royal Comfort, Heating, Air &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>edwardsroyalcomfort.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://edwardsroyalcomfort.com/lafayette-in/heat-pump-installation-replacement/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>info@edwardsroyalcomfort.com</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>765-323-4433</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Lafayette IN</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>90</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>heat pump installation Lafayette IN</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:52 UTC (cycle 58)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8554,7 +8554,6 @@
           <t>https://edwardsroyalcomfort.com/lafayette-in/heat-pump-installation-replacement/</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>info@edwardsroyalcomfort.com</t>
@@ -8584,6 +8583,66 @@
         </is>
       </c>
       <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Exteriors Plus LLC</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>exteriorsplusmn.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://exteriorsplusmn.com/roofers-bloomington-mn/</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Get Financing</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>general@exteriorsplusmn.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>952-345-3408</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Bloomington MN</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>100</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>roofing contractor Bloomington MN</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:53 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8648,6 +8648,66 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>South Side Home Improvement</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>southsidehomeimprovementllc.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://southsidehomeimprovementllc.com/roofing-repairs-wilmington-de/</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>South Side</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>info@southsidehomeimprovementllc.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>(302) 279-5669</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Wilmington DE</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>98</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>roof repair company Wilmington DE</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 20:56 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8708,6 +8708,62 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Flying Out Roofing</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>flyingoutroofing.net</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://www.flyingoutroofing.net/services/metal-roof/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>ty@flyingoutroofing.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>(405) 487-0183</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>98</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Edmond OK</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:05 UTC (cycle 67)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8729,7 +8729,6 @@
           <t>https://www.flyingoutroofing.net/services/metal-roof/</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>ty@flyingoutroofing.com</t>
@@ -8759,6 +8758,66 @@
         </is>
       </c>
       <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Martins HVAC Service</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>martinshvacservice.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://martinshvacservice.com/service-areas/pawtucket-ri/</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Star Rated</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>martinshvacservice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>401-692-4822</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Pawtucket RI</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>90</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>HVAC contractor Pawtucket RI</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:17 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8823,6 +8823,122 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Admiral Plumbing</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>admiralplumbing.com</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://www.admiralplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>(801) 960-4115</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Provo UT</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>100</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>plumbing company Provo UT</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Emergency Residential Plumbing &amp; HVAC Repair, Maintenance Contractor Orem &amp; Prov</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>berniesplumbingandheatingutah.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://www.berniesplumbingandheatingutah.com/</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Heating Co</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>climbingto360@gmail.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>(801) 373-7313</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Provo UT</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>88</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>plumbing company Provo UT</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:19 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8844,7 +8844,6 @@
           <t>https://www.admiralplumbing.com/</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
           <t>example@mysite.com</t>
@@ -8934,6 +8933,66 @@
         </is>
       </c>
       <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Lexington Roofing &amp; Remodeling</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>lexingtonroofingco.com</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://lexingtonroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>info@lexingtonroofingco.com</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>859-518-8175</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>100</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>roof repair company Lexington KY</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:21 UTC (cycle 78)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L147"/>
+  <dimension ref="A1:L148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8998,6 +8998,62 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Watts Heating</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>wattsheating.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://wattsheating.com/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>office@wattsheating.com</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>503-786-2858</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>90</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>heating and cooling company Portland OR</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:27 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9019,7 +9019,6 @@
           <t>https://wattsheating.com/</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>office@wattsheating.com</t>
@@ -9049,6 +9048,246 @@
         </is>
       </c>
       <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>24/7 Emergency Sewer &amp; Drain Service in Utica, NY | Utica Sewer Pros</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>uticasewerpros.com</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://uticasewerpros.com/</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Oneida County</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>hello@uticasewerpros.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>(315) 859-6204</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Utica NY</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>100</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>sewer repair Utica NY</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>King Roofing</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>kingroofco.com</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://www.kingroofco.com/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Hear From</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>admin@kingroofco.com</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>(385) 450-5464</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>100</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Orem UT</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>All Star Roofing LLC | Orem, UT</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>allstarroofpros.com</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://www.allstarroofpros.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>All Star</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>allstarroofingutah@gmail.com</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>(801) 381-0727</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>90</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Orem UT</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Riverway Plumbing and Mechanical</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>riverwayplumbing.com</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://riverwayplumbing.com/services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Riverway Plumbing</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>info@riverway-plumbing-and-mechanical-rroi.websitepro.hosting</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>(812) 327-8080</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>90</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>sewer repair Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:36 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9293,6 +9293,62 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Cullum Mechanical |</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>culluminc.com</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://culluminc.com/</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>info@culluminc.com</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>(843)-554-6645</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Charleston SC</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>90</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>HVAC contractor Charleston SC</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:37 UTC (cycle 89)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9314,7 +9314,6 @@
           <t>https://culluminc.com/</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
           <t>info@culluminc.com</t>
@@ -9344,6 +9343,66 @@
         </is>
       </c>
       <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Premium Plumbing</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>mypremiumplumbing.com</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://mypremiumplumbing.com/water-heater-repair-in-clearwater-fl/</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Google Reviews</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>service@mypremiumplumbing.com</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>813-773-6486</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>100</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>water heater repair Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:45 UTC (cycle 94)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9408,6 +9408,62 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Grand Prairie Water Heater</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>waterheatersrepairtx.com</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://waterheatersrepairtx.com/water-heater-grand-prairie.html</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>service@waterheatersrepairtx.com</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>346-439-5329</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>70</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>water heater repair Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:55 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L155"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9429,7 +9429,6 @@
           <t>https://waterheatersrepairtx.com/water-heater-grand-prairie.html</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>service@waterheatersrepairtx.com</t>
@@ -9459,6 +9458,62 @@
         </is>
       </c>
       <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Sewer &amp; Drain Cleaning | Tuscaloosa, AL</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>turnerplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://www.turnerplumbinginc.com/sewer-drain-cleaning-slab-leak-repair</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>info@turnerplumbinginc.net</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>(205) 345-4825</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>100</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>sewer repair Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-16 21:56 UTC (cycle 102)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-16.xlsx
+++ b/output/leads_2026-09-16.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9484,7 +9484,6 @@
           <t>https://www.turnerplumbinginc.com/sewer-drain-cleaning-slab-leak-repair</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
           <t>info@turnerplumbinginc.net</t>
@@ -9514,6 +9513,62 @@
         </is>
       </c>
       <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Boyd's Custom Remodeling Inc</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>boydscustomremodeling.com</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://www.boydscustomremodeling.com/roofing-installation-in-dover-de/</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>%20boyd.kevin1978@gmail.com</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>302-222-2322</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Dover DE</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>100</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>roof replacement Dover DE</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>

</xml_diff>